<commit_message>
feat(quote-to-order): thêm cột "Kho yêu cầu" (Hà Nội | Hồ Chí Minh)
Mẫu Base mới 14 cột: thêm "Kho yêu cầu (*)" ở cuối, bắt buộc.
- Tự nhận diện cột trong báo giá, chuẩn hóa giá trị (HN/HCM, không dấu);
  không có cột hoặc giá trị lạ thì để trống, người dùng chọn trên bảng.
- Chặn tải khi dòng đã chọn thiếu kho; server kiểm tra lại.
- Tổng quát hóa trường lựa chọn (Loại hàng, Kho yêu cầu); ghép cột đã nhớ
  vẫn dùng được với trường mới.
- Thay file mẫu đơn hàng bằng bản 14 cột của PO.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/quote_to_order/bang-hang-hoa_template.xlsx
+++ b/assets/quote_to_order/bang-hang-hoa_template.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="14">
   <si>
     <t>Tên hàng (*)</t>
   </si>
@@ -55,6 +55,9 @@
   </si>
   <si>
     <t>Ghi chú khác</t>
+  </si>
+  <si>
+    <t>Kho yêu cầu (*)</t>
   </si>
 </sst>
 </file>
@@ -411,7 +414,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="true" style="0"/>
@@ -427,9 +430,10 @@
     <col min="11" max="11" width="20" customWidth="true" style="0"/>
     <col min="12" max="12" width="20" customWidth="true" style="0"/>
     <col min="13" max="13" width="20" customWidth="true" style="0"/>
+    <col min="14" max="14" width="20" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -468,6 +472,9 @@
       </c>
       <c r="M1" s="1" t="s">
         <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>